<commit_message>
fix: modify task setting of topical chat
</commit_message>
<xml_diff>
--- a/outputs/llm_eval/topical_yjx/mul/two_turns/correlation_results.xlsx
+++ b/outputs/llm_eval/topical_yjx/mul/two_turns/correlation_results.xlsx
@@ -417,13 +417,13 @@
         <v>4</v>
       </c>
       <c r="B2">
-        <v>0.424770241485801</v>
+        <v>0.441336173767255</v>
       </c>
       <c r="C2">
-        <v>0.4365772976202504</v>
+        <v>0.4313950753026501</v>
       </c>
       <c r="D2">
-        <v>0.3752080070223991</v>
+        <v>0.3963789817294336</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -431,13 +431,13 @@
         <v>5</v>
       </c>
       <c r="B3">
-        <v>0.5009370850281214</v>
+        <v>0.5000721833833485</v>
       </c>
       <c r="C3">
-        <v>0.4842646933689271</v>
+        <v>0.50105055287608</v>
       </c>
       <c r="D3">
-        <v>0.4529619607967388</v>
+        <v>0.4542638674868268</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -445,13 +445,13 @@
         <v>6</v>
       </c>
       <c r="B4">
-        <v>0.6758646620024861</v>
+        <v>0.6641075896917169</v>
       </c>
       <c r="C4">
-        <v>0.6759812098656722</v>
+        <v>0.6655064595791578</v>
       </c>
       <c r="D4">
-        <v>0.6091778333472455</v>
+        <v>0.6067006699620727</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -459,13 +459,13 @@
         <v>7</v>
       </c>
       <c r="B5">
-        <v>0.5572311262851002</v>
+        <v>0.6020714965050338</v>
       </c>
       <c r="C5">
-        <v>0.5703087953893557</v>
+        <v>0.617079539439147</v>
       </c>
       <c r="D5">
-        <v>0.5399999805776442</v>
+        <v>0.5826140031632374</v>
       </c>
     </row>
   </sheetData>

</xml_diff>